<commit_message>
lan date update, regional forecasting logic update
</commit_message>
<xml_diff>
--- a/Region_results/Region_Forecasting_26_0603_0609.xlsx
+++ b/Region_results/Region_Forecasting_26_0603_0609.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lena/forecasting_new_backup/Region_results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lena/forecasting_new/Region_results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED0A67B3-867C-3A45-949B-ACEC7CF12809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36AFEFFE-C388-C940-9BCF-4F278C6D44AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -255,7 +255,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -320,7 +320,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -625,6 +625,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D505"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">

</xml_diff>